<commit_message>
Update: Documentação iniciada. Feito 'Resumo' & 'Introdução'
</commit_message>
<xml_diff>
--- a/results/evaluation_v3/excel/comparacao_modelos.xlsx
+++ b/results/evaluation_v3/excel/comparacao_modelos.xlsx
@@ -1,23 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guilherme\Desktop\6º Semestre\TCC\results\evaluation_v3\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B660EF42-80DC-4E5A-AF7F-24401F75F316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD3067F-22D8-45EA-8D83-AFCAA52A51B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Comparação de Modelos" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,15 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Model</t>
   </si>
   <si>
     <t>Accuracy</t>
-  </si>
-  <si>
-    <t>Accuracy (mean ± std)</t>
   </si>
   <si>
     <t>Precision (Macro Avg)</t>
@@ -59,7 +53,22 @@
     <t>F1-Score (Macro Avg)</t>
   </si>
   <si>
-    <t>F1-Score (mean ± std)</t>
+    <t>MobileNetV3Large</t>
+  </si>
+  <si>
+    <t>MobileNetV3Small</t>
+  </si>
+  <si>
+    <t>EfficientNetV2B3</t>
+  </si>
+  <si>
+    <t>DenseNet121</t>
+  </si>
+  <si>
+    <t>EfficientNetV2B0</t>
+  </si>
+  <si>
+    <t>ResNet50V2</t>
   </si>
 </sst>
 </file>
@@ -130,47 +139,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <font>
         <b val="0"/>
@@ -424,19 +393,19 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>EfficientNetV2B0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>EfficientNetV2B3</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>MobileNetV3Large</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>MobileNetV3Small</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>EfficientNetV2B3</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>DenseNet121</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>EfficientNetV2B0</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>ResNet50V2</c:v>
@@ -451,19 +420,19 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>0.98579295154185009</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.98573788546255492</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>0.97984581497797352</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>0.97797356828193838</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.98573788546255492</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>0.97604625550660806</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.98579295154185009</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.95280837004405294</c:v>
@@ -507,19 +476,19 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>EfficientNetV2B0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>EfficientNetV2B3</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>MobileNetV3Large</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>MobileNetV3Small</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>EfficientNetV2B3</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>DenseNet121</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>EfficientNetV2B0</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>ResNet50V2</c:v>
@@ -534,19 +503,19 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>0.98225456204086581</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.98216362818972325</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>0.97506131227955861</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>0.97033820799808868</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.98216362818972325</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>0.96992324824472931</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.98225456204086581</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.93912382709307685</c:v>
@@ -590,19 +559,19 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>EfficientNetV2B0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>EfficientNetV2B3</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>MobileNetV3Large</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>MobileNetV3Small</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>EfficientNetV2B3</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>DenseNet121</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>EfficientNetV2B0</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>ResNet50V2</c:v>
@@ -617,19 +586,19 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>0.98132848476120116</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.98065587371266683</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>0.97356497246705642</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>0.97046499022164667</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.98065587371266683</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>0.96974465387112763</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.98132848476120116</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.93522548478357392</c:v>
@@ -673,19 +642,19 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>EfficientNetV2B0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>EfficientNetV2B3</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>MobileNetV3Large</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>MobileNetV3Small</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>EfficientNetV2B3</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>DenseNet121</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>EfficientNetV2B0</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>ResNet50V2</c:v>
@@ -700,19 +669,19 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>0.98175130098541907</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.98134813272746391</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>0.97423869936284146</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>0.97035232329688303</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.98134813272746391</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>0.96975912502650419</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.98175130098541907</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.93699038639945653</c:v>
@@ -1516,190 +1485,18 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="FOLDS"/>
-      <sheetName val="MEDIA_FOLD"/>
-      <sheetName val="CONFIGURACAO"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>MobileNetV3Large</v>
-          </cell>
-          <cell r="B2">
-            <v>0.97984581497797352</v>
-          </cell>
-          <cell r="C2">
-            <v>2.2146561180826181E-3</v>
-          </cell>
-          <cell r="D2">
-            <v>0.97506131227955861</v>
-          </cell>
-          <cell r="F2">
-            <v>0.97356497246705642</v>
-          </cell>
-          <cell r="H2">
-            <v>0.97423869936284146</v>
-          </cell>
-          <cell r="I2">
-            <v>2.8661773392239498E-3</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>MobileNetV3Small</v>
-          </cell>
-          <cell r="B3">
-            <v>0.97797356828193838</v>
-          </cell>
-          <cell r="C3">
-            <v>8.7067116194064866E-4</v>
-          </cell>
-          <cell r="D3">
-            <v>0.97033820799808868</v>
-          </cell>
-          <cell r="F3">
-            <v>0.97046499022164667</v>
-          </cell>
-          <cell r="H3">
-            <v>0.97035232329688303</v>
-          </cell>
-          <cell r="I3">
-            <v>1.5526161478284621E-3</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>EfficientNetV2B3</v>
-          </cell>
-          <cell r="B4">
-            <v>0.98573788546255492</v>
-          </cell>
-          <cell r="C4">
-            <v>2.0456140551769562E-3</v>
-          </cell>
-          <cell r="D4">
-            <v>0.98216362818972325</v>
-          </cell>
-          <cell r="F4">
-            <v>0.98065587371266683</v>
-          </cell>
-          <cell r="H4">
-            <v>0.98134813272746391</v>
-          </cell>
-          <cell r="I4">
-            <v>3.1521990742292639E-3</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>DenseNet121</v>
-          </cell>
-          <cell r="B5">
-            <v>0.97604625550660806</v>
-          </cell>
-          <cell r="C5">
-            <v>2.3684816263883808E-3</v>
-          </cell>
-          <cell r="D5">
-            <v>0.96992324824472931</v>
-          </cell>
-          <cell r="F5">
-            <v>0.96974465387112763</v>
-          </cell>
-          <cell r="H5">
-            <v>0.96975912502650419</v>
-          </cell>
-          <cell r="I5">
-            <v>3.5569903041252939E-3</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>EfficientNetV2B0</v>
-          </cell>
-          <cell r="B6">
-            <v>0.98579295154185009</v>
-          </cell>
-          <cell r="C6">
-            <v>2.31670528281526E-3</v>
-          </cell>
-          <cell r="D6">
-            <v>0.98225456204086581</v>
-          </cell>
-          <cell r="F6">
-            <v>0.98132848476120116</v>
-          </cell>
-          <cell r="H6">
-            <v>0.98175130098541907</v>
-          </cell>
-          <cell r="I6">
-            <v>2.8772932512907438E-3</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>ResNet50V2</v>
-          </cell>
-          <cell r="B7">
-            <v>0.95280837004405294</v>
-          </cell>
-          <cell r="C7">
-            <v>3.0819791451444341E-3</v>
-          </cell>
-          <cell r="D7">
-            <v>0.93912382709307685</v>
-          </cell>
-          <cell r="F7">
-            <v>0.93522548478357392</v>
-          </cell>
-          <cell r="H7">
-            <v>0.93699038639945653</v>
-          </cell>
-          <cell r="I7">
-            <v>4.4758047709830152E-3</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ECD4892B-38C2-46BF-B65A-7B1CBB8BB7C3}" name="Tabela1" displayName="Tabela1" ref="C3:I9" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="C3:I9" xr:uid="{ECD4892B-38C2-46BF-B65A-7B1CBB8BB7C3}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{1F68EB1E-1D37-4556-8033-DA1AF235CD55}" name="Model" dataDxfId="6">
-      <calculatedColumnFormula>[1]MEDIA_FOLD!A2</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="20" xr3:uid="{ABC9E850-E400-4BA6-9404-EF2A36410D2E}" name="Accuracy" dataDxfId="5">
-      <calculatedColumnFormula>[1]MEDIA_FOLD!B2</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="19" xr3:uid="{26C8949D-71D0-4E9D-9676-7348C26EC062}" name="Precision (Macro Avg)" dataDxfId="4">
-      <calculatedColumnFormula>[1]MEDIA_FOLD!D2</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="18" xr3:uid="{AA5397E3-CD8C-4C66-9D17-53247A8FC39E}" name="Recall (Macro Avg)" dataDxfId="3">
-      <calculatedColumnFormula>[1]MEDIA_FOLD!F2</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="17" xr3:uid="{1D199753-E081-4FA1-B186-881131937094}" name="F1-Score (Macro Avg)" dataDxfId="2">
-      <calculatedColumnFormula>[1]MEDIA_FOLD!H2</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{5EBB0357-ECA6-4128-8D59-FA86E8016AAD}" name="Accuracy (mean ± std)" dataDxfId="1">
-      <calculatedColumnFormula>TEXT([1]MEDIA_FOLD!B2, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!C2, "0,0000")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{B358297F-18F5-428D-BE67-539F783D331C}" name="F1-Score (mean ± std)" dataDxfId="0">
-      <calculatedColumnFormula>TEXT([1]MEDIA_FOLD!H2, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!I2, "0,0000")</calculatedColumnFormula>
-    </tableColumn>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ECD4892B-38C2-46BF-B65A-7B1CBB8BB7C3}" name="Tabela1" displayName="Tabela1" ref="C3:G9" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="C3:G9" xr:uid="{ECD4892B-38C2-46BF-B65A-7B1CBB8BB7C3}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C4:G9">
+    <sortCondition descending="1" ref="D3:D9"/>
+  </sortState>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{1F68EB1E-1D37-4556-8033-DA1AF235CD55}" name="Model" dataDxfId="4"/>
+    <tableColumn id="20" xr3:uid="{ABC9E850-E400-4BA6-9404-EF2A36410D2E}" name="Accuracy" dataDxfId="3"/>
+    <tableColumn id="19" xr3:uid="{26C8949D-71D0-4E9D-9676-7348C26EC062}" name="Precision (Macro Avg)" dataDxfId="2"/>
+    <tableColumn id="18" xr3:uid="{AA5397E3-CD8C-4C66-9D17-53247A8FC39E}" name="Recall (Macro Avg)" dataDxfId="1"/>
+    <tableColumn id="17" xr3:uid="{1D199753-E081-4FA1-B186-881131937094}" name="F1-Score (Macro Avg)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1969,16 +1766,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="C3:I9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="4" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="22.6640625" customWidth="1"/>
     <col min="5" max="5" width="34" customWidth="1"/>
-    <col min="6" max="6" width="30.28515625" customWidth="1"/>
-    <col min="7" max="7" width="34.7109375" customWidth="1"/>
-    <col min="8" max="9" width="36.85546875" customWidth="1"/>
+    <col min="6" max="6" width="30.33203125" customWidth="1"/>
+    <col min="7" max="7" width="34.6640625" customWidth="1"/>
+    <col min="8" max="9" width="36.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1986,200 +1783,130 @@
         <v>1</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.98579295154185009</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0.98225456204086581</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.98132848476120116</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0.98175130098541907</v>
+      </c>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.98573788546255492</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.98216362818972325</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.98065587371266683</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0.98134813272746391</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="I3" s="3" t="s">
+      <c r="D6" s="2">
+        <v>0.97984581497797352</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0.97506131227955861</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.97356497246705642</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.97423869936284146</v>
+      </c>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="D7" s="2">
+        <v>0.97797356828193838</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0.97033820799808868</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0.97046499022164667</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0.97035232329688303</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
     </row>
-    <row r="4" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="1" t="str">
-        <f>[1]MEDIA_FOLD!A2</f>
-        <v>MobileNetV3Large</v>
-      </c>
-      <c r="D4" s="2">
-        <f>[1]MEDIA_FOLD!B2</f>
-        <v>0.97984581497797352</v>
-      </c>
-      <c r="E4" s="2">
-        <f>[1]MEDIA_FOLD!D2</f>
-        <v>0.97506131227955861</v>
-      </c>
-      <c r="F4" s="2">
-        <f>[1]MEDIA_FOLD!F2</f>
-        <v>0.97356497246705642</v>
-      </c>
-      <c r="G4" s="2">
-        <f>[1]MEDIA_FOLD!H2</f>
-        <v>0.97423869936284146</v>
-      </c>
-      <c r="H4" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!B2, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!C2, "0,0000")</f>
-        <v>0,9798 ± 0,0022</v>
-      </c>
-      <c r="I4" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!H2, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!I2, "0,0000")</f>
-        <v>0,9742 ± 0,0029</v>
-      </c>
+    <row r="8" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0.97604625550660806</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0.96992324824472931</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.96974465387112763</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.96975912502650419</v>
+      </c>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
     </row>
-    <row r="5" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="1" t="str">
-        <f>[1]MEDIA_FOLD!A3</f>
-        <v>MobileNetV3Small</v>
-      </c>
-      <c r="D5" s="2">
-        <f>[1]MEDIA_FOLD!B3</f>
-        <v>0.97797356828193838</v>
-      </c>
-      <c r="E5" s="2">
-        <f>[1]MEDIA_FOLD!D3</f>
-        <v>0.97033820799808868</v>
-      </c>
-      <c r="F5" s="2">
-        <f>[1]MEDIA_FOLD!F3</f>
-        <v>0.97046499022164667</v>
-      </c>
-      <c r="G5" s="2">
-        <f>[1]MEDIA_FOLD!H3</f>
-        <v>0.97035232329688303</v>
-      </c>
-      <c r="H5" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!B3, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!C3, "0,0000")</f>
-        <v>0,9780 ± 0,0009</v>
-      </c>
-      <c r="I5" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!H3, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!I3, "0,0000")</f>
-        <v>0,9704 ± 0,0016</v>
-      </c>
-    </row>
-    <row r="6" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="1" t="str">
-        <f>[1]MEDIA_FOLD!A4</f>
-        <v>EfficientNetV2B3</v>
-      </c>
-      <c r="D6" s="2">
-        <f>[1]MEDIA_FOLD!B4</f>
-        <v>0.98573788546255492</v>
-      </c>
-      <c r="E6" s="2">
-        <f>[1]MEDIA_FOLD!D4</f>
-        <v>0.98216362818972325</v>
-      </c>
-      <c r="F6" s="2">
-        <f>[1]MEDIA_FOLD!F4</f>
-        <v>0.98065587371266683</v>
-      </c>
-      <c r="G6" s="2">
-        <f>[1]MEDIA_FOLD!H4</f>
-        <v>0.98134813272746391</v>
-      </c>
-      <c r="H6" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!B4, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!C4, "0,0000")</f>
-        <v>0,9857 ± 0,0020</v>
-      </c>
-      <c r="I6" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!H4, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!I4, "0,0000")</f>
-        <v>0,9813 ± 0,0032</v>
-      </c>
-    </row>
-    <row r="7" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="1" t="str">
-        <f>[1]MEDIA_FOLD!A5</f>
-        <v>DenseNet121</v>
-      </c>
-      <c r="D7" s="2">
-        <f>[1]MEDIA_FOLD!B5</f>
-        <v>0.97604625550660806</v>
-      </c>
-      <c r="E7" s="2">
-        <f>[1]MEDIA_FOLD!D5</f>
-        <v>0.96992324824472931</v>
-      </c>
-      <c r="F7" s="2">
-        <f>[1]MEDIA_FOLD!F5</f>
-        <v>0.96974465387112763</v>
-      </c>
-      <c r="G7" s="2">
-        <f>[1]MEDIA_FOLD!H5</f>
-        <v>0.96975912502650419</v>
-      </c>
-      <c r="H7" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!B5, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!C5, "0,0000")</f>
-        <v>0,9760 ± 0,0024</v>
-      </c>
-      <c r="I7" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!H5, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!I5, "0,0000")</f>
-        <v>0,9698 ± 0,0036</v>
-      </c>
-    </row>
-    <row r="8" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="1" t="str">
-        <f>[1]MEDIA_FOLD!A6</f>
-        <v>EfficientNetV2B0</v>
-      </c>
-      <c r="D8" s="2">
-        <f>[1]MEDIA_FOLD!B6</f>
-        <v>0.98579295154185009</v>
-      </c>
-      <c r="E8" s="2">
-        <f>[1]MEDIA_FOLD!D6</f>
-        <v>0.98225456204086581</v>
-      </c>
-      <c r="F8" s="2">
-        <f>[1]MEDIA_FOLD!F6</f>
-        <v>0.98132848476120116</v>
-      </c>
-      <c r="G8" s="2">
-        <f>[1]MEDIA_FOLD!H6</f>
-        <v>0.98175130098541907</v>
-      </c>
-      <c r="H8" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!B6, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!C6, "0,0000")</f>
-        <v>0,9858 ± 0,0023</v>
-      </c>
-      <c r="I8" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!H6, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!I6, "0,0000")</f>
-        <v>0,9818 ± 0,0029</v>
-      </c>
-    </row>
-    <row r="9" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="1" t="str">
-        <f>[1]MEDIA_FOLD!A7</f>
-        <v>ResNet50V2</v>
+    <row r="9" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="D9" s="2">
-        <f>[1]MEDIA_FOLD!B7</f>
         <v>0.95280837004405294</v>
       </c>
       <c r="E9" s="2">
-        <f>[1]MEDIA_FOLD!D7</f>
         <v>0.93912382709307685</v>
       </c>
       <c r="F9" s="2">
-        <f>[1]MEDIA_FOLD!F7</f>
         <v>0.93522548478357392</v>
       </c>
       <c r="G9" s="2">
-        <f>[1]MEDIA_FOLD!H7</f>
         <v>0.93699038639945653</v>
       </c>
-      <c r="H9" s="4" t="str">
-        <f>TEXT([1]MEDIA_FOLD!B7, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!C7, "0,0000")</f>
-        <v>0,9528 ± 0,0031</v>
-      </c>
-      <c r="I9" s="1" t="str">
-        <f>TEXT([1]MEDIA_FOLD!H7, "0,0000") &amp; " ± " &amp; TEXT([1]MEDIA_FOLD!I7, "0,0000")</f>
-        <v>0,9370 ± 0,0045</v>
-      </c>
+      <c r="H9" s="4"/>
+      <c r="I9" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update: Modelos testados com tamanho menor da imagem de entrada e atualização da documentação (Monografia)
</commit_message>
<xml_diff>
--- a/results/evaluation_v3/excel/comparacao_modelos.xlsx
+++ b/results/evaluation_v3/excel/comparacao_modelos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guilherme\Desktop\6º Semestre\TCC\results\evaluation_v3\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD3067F-22D8-45EA-8D83-AFCAA52A51B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F719678A-F351-4A31-A72E-97AC9A1196B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>Model</t>
   </si>
   <si>
-    <t>Accuracy</t>
-  </si>
-  <si>
     <t>Precision (Macro Avg)</t>
   </si>
   <si>
@@ -69,6 +66,9 @@
   </si>
   <si>
     <t>ResNet50V2</t>
+  </si>
+  <si>
+    <t>Acurácia</t>
   </si>
 </sst>
 </file>
@@ -109,7 +109,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -117,11 +117,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -133,6 +148,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -219,6 +243,26 @@
       </font>
       <numFmt numFmtId="164" formatCode="0.0000"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -239,6 +283,26 @@
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -372,7 +436,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Accuracy</c:v>
+                  <c:v>Acurácia</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -420,7 +484,7 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.98579295154185009</c:v>
+                  <c:v>0.98579295154184998</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.98573788546255492</c:v>
@@ -503,7 +567,7 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.98225456204086581</c:v>
+                  <c:v>0.98225456204086603</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.98216362818972325</c:v>
@@ -1493,7 +1557,7 @@
   </sortState>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{1F68EB1E-1D37-4556-8033-DA1AF235CD55}" name="Model" dataDxfId="4"/>
-    <tableColumn id="20" xr3:uid="{ABC9E850-E400-4BA6-9404-EF2A36410D2E}" name="Accuracy" dataDxfId="3"/>
+    <tableColumn id="20" xr3:uid="{ABC9E850-E400-4BA6-9404-EF2A36410D2E}" name="Acurácia" dataDxfId="3"/>
     <tableColumn id="19" xr3:uid="{26C8949D-71D0-4E9D-9676-7348C26EC062}" name="Precision (Macro Avg)" dataDxfId="2"/>
     <tableColumn id="18" xr3:uid="{AA5397E3-CD8C-4C66-9D17-53247A8FC39E}" name="Recall (Macro Avg)" dataDxfId="1"/>
     <tableColumn id="17" xr3:uid="{1D199753-E081-4FA1-B186-881131937094}" name="F1-Score (Macro Avg)" dataDxfId="0"/>
@@ -1769,40 +1833,40 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="4" width="22.6640625" customWidth="1"/>
-    <col min="5" max="5" width="34" customWidth="1"/>
-    <col min="6" max="6" width="30.33203125" customWidth="1"/>
-    <col min="7" max="7" width="34.6640625" customWidth="1"/>
+    <col min="5" max="5" width="30.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="36.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>4</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
     </row>
     <row r="4" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.98579295154185009</v>
+      <c r="C4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="7">
+        <v>0.98579295154184998</v>
       </c>
       <c r="E4" s="2">
-        <v>0.98225456204086581</v>
+        <v>0.98225456204086603</v>
       </c>
       <c r="F4" s="2">
         <v>0.98132848476120116</v>
@@ -1814,10 +1878,10 @@
       <c r="I4" s="1"/>
     </row>
     <row r="5" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="2">
+      <c r="C5" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="7">
         <v>0.98573788546255492</v>
       </c>
       <c r="E5" s="2">
@@ -1833,10 +1897,10 @@
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="2">
+      <c r="C6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="7">
         <v>0.97984581497797352</v>
       </c>
       <c r="E6" s="2">
@@ -1852,10 +1916,10 @@
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="2">
+      <c r="C7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="7">
         <v>0.97797356828193838</v>
       </c>
       <c r="E7" s="2">
@@ -1871,10 +1935,10 @@
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="2">
+      <c r="C8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="7">
         <v>0.97604625550660806</v>
       </c>
       <c r="E8" s="2">
@@ -1890,10 +1954,10 @@
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="3:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="2">
+      <c r="C9" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="7">
         <v>0.95280837004405294</v>
       </c>
       <c r="E9" s="2">

</xml_diff>